<commit_message>
Add validators and semantic analysis for input data
- Introduced new validation functions in `text_validator.py` to check for empty values, length constraints, invalid characters, and semantic similarity.
- Implemented a semantic validation mechanism using `SentenceTransformer` in `semantic_validator.py` to assess the similarity of input text against a predefined catalog.
- Created a `vector_validator.py` to handle specific validation logic for vector data, including checks for numeric values and semantic validation.
- Added constants for capital sources, location factors, and decision-makers in `catalogs.py`.
- Compiled a list of common invalid text patterns in `text_validator.py`.
- Generated new cache files for compiled Python modules.
- Added an Excel file placeholder for future data integration.
</commit_message>
<xml_diff>
--- a/Vaciado_ENAPROCE2026.xlsx
+++ b/Vaciado_ENAPROCE2026.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\cristina.sanchez\Documents\VALIDACION_VECTORES\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\martin.macias\Downloads\VALIDACION_VECTORES\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E4D06494-1F1F-45ED-9B74-9ED1F13A5E4B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{684255A6-5006-4333-B1CA-3B6D229A1C68}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3396" uniqueCount="834">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3400" uniqueCount="838">
   <si>
     <t>ID_MUESTRA</t>
   </si>
@@ -2531,13 +2531,25 @@
   </si>
   <si>
     <t>holiholiholihollllllllll</t>
+  </si>
+  <si>
+    <t>Propios</t>
+  </si>
+  <si>
+    <t>sdlfmsgmomsv</t>
+  </si>
+  <si>
+    <t>Hola buen dí</t>
+  </si>
+  <si>
+    <t>hola</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2">
+  <fonts count="3">
     <font>
       <sz val="11"/>
       <color indexed="8"/>
@@ -2548,6 +2560,14 @@
     <font>
       <sz val="11"/>
       <name val="Dialog"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color indexed="8"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="2">
@@ -2570,7 +2590,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
@@ -2579,6 +2599,7 @@
     <xf numFmtId="49" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="right" vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="49" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -2916,7 +2937,11 @@
   <dimension ref="A1:MA13"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="16384" width="11.5546875" style="1"/>
+    <col min="1" max="10" width="11.5546875" style="1"/>
+    <col min="11" max="11" width="39.88671875" style="1" customWidth="1"/>
+    <col min="12" max="16" width="11.5546875" style="1"/>
+    <col min="17" max="17" width="34.33203125" style="1" customWidth="1"/>
+    <col min="18" max="16384" width="11.5546875" style="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:339">
@@ -3969,8 +3994,11 @@
       <c r="J2" s="1" t="s">
         <v>592</v>
       </c>
+      <c r="K2" s="1" t="s">
+        <v>595</v>
+      </c>
       <c r="L2" s="1" t="s">
-        <v>592</v>
+        <v>590</v>
       </c>
       <c r="M2" s="1" t="s">
         <v>593</v>
@@ -5353,8 +5381,11 @@
       <c r="J4" s="1" t="s">
         <v>592</v>
       </c>
+      <c r="K4" s="1" t="s">
+        <v>835</v>
+      </c>
       <c r="L4" s="1" t="s">
-        <v>592</v>
+        <v>589</v>
       </c>
       <c r="M4" s="1" t="s">
         <v>593</v>
@@ -5827,7 +5858,10 @@
         <v>591</v>
       </c>
       <c r="T5" s="1" t="s">
-        <v>594</v>
+        <v>647</v>
+      </c>
+      <c r="U5" s="1" t="s">
+        <v>837</v>
       </c>
       <c r="V5" s="1" t="s">
         <v>595</v>
@@ -6503,8 +6537,8 @@
       <c r="J6" s="1" t="s">
         <v>590</v>
       </c>
-      <c r="K6" s="1" t="s">
-        <v>377</v>
+      <c r="K6" s="4" t="s">
+        <v>836</v>
       </c>
       <c r="L6" s="1" t="s">
         <v>627</v>
@@ -6530,7 +6564,7 @@
       <c r="T6" s="1" t="s">
         <v>647</v>
       </c>
-      <c r="U6" s="1" t="s">
+      <c r="U6" s="4" t="s">
         <v>377</v>
       </c>
       <c r="V6" s="1" t="s">
@@ -7899,7 +7933,7 @@
       <c r="J8" s="1" t="s">
         <v>592</v>
       </c>
-      <c r="K8" s="1" t="s">
+      <c r="K8" s="4" t="s">
         <v>390</v>
       </c>
       <c r="L8" s="1" t="s">
@@ -8731,6 +8765,9 @@
       </c>
       <c r="J9" s="1" t="s">
         <v>599</v>
+      </c>
+      <c r="K9" s="1" t="s">
+        <v>834</v>
       </c>
       <c r="L9" s="1" t="s">
         <v>592</v>

</xml_diff>